<commit_message>
chore: migra use_container_width->width y regenera plantillas al esquema real
- pages/*: use_container_width -> width='stretch' (sin deprecaciones de Streamlit).
- data/templates/*: regeneradas para coincidir con el esquema que lee data_loader.
- tools/generar_plantillas.py: generador reproducible de plantillas.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/templates/CONTEXTO_TERRITORIAL.xlsx
+++ b/data/templates/CONTEXTO_TERRITORIAL.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,26 +25,16 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00667eea"/>
-        <bgColor rgb="00667eea"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -52,20 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -433,237 +415,174 @@
   </sheetPr>
   <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Indicador</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Nombre</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Unidad</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Año</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Comp_Nacional</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Pobreza Multidimensional</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Pobreza Multidimensional</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>67</v>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Pobreza multidimensional</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>DANE</t>
         </is>
       </c>
-      <c r="F2" s="2" t="n">
-        <v>2024</v>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>11.5</v>
-      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Informalidad</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Tasa de informalidad</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>83</v>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Tasa de informalidad laboral</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>DANE-GEIH</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Educacion Promedio</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Años promedio de escolaridad</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>años</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Admvo. Mpal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Acceso Internet</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Cobertura hogares con internet</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>MinTIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Desempleo Juvenil</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Desempleo &lt; 25 años</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>DANE</t>
         </is>
       </c>
-      <c r="F3" s="2" t="n">
-        <v>2024</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Educacion Promedio</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Años promedio</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>años</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Administrativo</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>2023</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>10.1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Acceso Internet</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Cobertura hogar</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Participacion Ciudadana</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Participación en espacios cívicos</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>MinTIC</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>2024</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Desempleo Juvenil</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Tasa &lt; 25 años</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>DANE</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>2024</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Participacion Ciudadana</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Participación</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Administrativo</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>2023</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>15</v>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Admvo. Mpal.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>